<commit_message>
Yayin: is plani B2 sablonuna gore yeniden yazildi (6 donem, 36.000 adet)
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
+++ b/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
@@ -708,10 +708,10 @@
         <v>36000</v>
       </c>
       <c r="C19" s="8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>252000</v>
+        <v>216000</v>
       </c>
     </row>
     <row r="20" ht="26" customHeight="1">
@@ -750,7 +750,7 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>610.000 kg</t>
+          <t>523.000 kg</t>
         </is>
       </c>
       <c r="C24" s="5" t="n"/>
@@ -759,7 +759,7 @@
     <row r="25" ht="26" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>36.000 adet/dönem x 7 dönem x %96 yaşama gücü x 2,52 kg kesim ağırlığı.</t>
+          <t>36.000 adet/dönem x 6 dönem x %96 yaşama gücü x 2,52 kg kesim ağırlığı.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: kapasite 36.000 adet/dönem izleri temizlendi
Teknik projede "15 adet/m²" bayat yoğunluğu ile A6 ve teknik projedeki
noktalı "16.97" yazımı düzeltildi; yayın sayfasının teknik proje
açıklaması kaynaktan üretiliyor.

Keşif değişmedi: uygun harcama 15.774.454,50 TL = 298.994 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
+++ b/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
@@ -717,7 +717,7 @@
     <row r="20" ht="26" customHeight="1">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>2 kümes x 1.060,42 m² iç alan = 2.120,84 m²; 16.97 adet/m² yoğunluk (rehberin 13-17 adet/m² aralığındadır).</t>
+          <t>2 kümes x 1.060,42 m² iç alan = 2.120,84 m²; 16,97 adet/m² yoğunluk (rehberin 13-17 adet/m² aralığındadır).</t>
         </is>
       </c>
     </row>
@@ -1031,7 +1031,7 @@
       </c>
       <c r="G5" s="4" t="inlineStr">
         <is>
-          <t>Kapasiteler kümesin kendi ölçüsünden çıkar: 78,55 x 13,50 m iç alan, 15 adet/m² yoğunluk. Yemleme 3 hat, sulama 4 hat; tünel fan debisi 2,50 m/sn hava hızına, ped alanı ve klape sayısı aynı debiye göre seçilmiştir. Isıtma kapasitesi kümesin ısı yükü hesabından gelir. Adetler mekanik projeden gelir: kümes başına 46.717 m³/h hava debisi için 4 tünel fanı ve 30 klape (30 x 1.750 = 52.500 m³/h). Yerleşim planı bu adetlerle çizilecektir.</t>
+          <t>Kapasiteler kümesin kendi ölçüsünden çıkar: 78,55 x 13,50 m iç alan, 16,97 adet/m² yoğunluk ile kümes başına 18.000 adet/dönem. Yemleme 3 hat, sulama 4 hat; tünel fan debisi 2,50 m/sn hava hızına, ped alanı ve klape sayısı aynı debiye göre seçilmiştir. Isıtma kapasitesi kümesin ısı yükü hesabından gelir. Adetler mekanik projeden gelir: kümes başına 46.717 m³/h hava debisi için 4 tünel fanı ve 30 klape (30 x 1.750 = 52.500 m³/h). Yerleşim planı bu adetlerle çizilecektir.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Yayın: altlık 57 ton, yakıt 51 ton — 6 döneme göre güncellendi
Keşif değişmedi: uygun harcama 15.774.454,50 TL = 298.994 Avro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HJPp6bx7wepUX5p8fxGcjg
</commit_message>
<xml_diff>
--- a/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
+++ b/belgeler/44_TEKNIK_PROJE_TP1013.xlsx
@@ -792,7 +792,7 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>66 ton</t>
+          <t>57 ton</t>
         </is>
       </c>
       <c r="C29" s="5" t="n"/>
@@ -806,7 +806,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>60 ton</t>
+          <t>51 ton</t>
         </is>
       </c>
       <c r="C30" s="5" t="n"/>

</xml_diff>